<commit_message>
fix excel BBGN Thep long
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC1_BBGN_ThepLong.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC1_BBGN_ThepLong.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7F04E9-7FAC-4E16-BFDB-DB97A07E307A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05E55899-F6AE-4946-8BD7-C5560080824E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>STT</t>
   </si>
@@ -40,50 +40,44 @@
     <t>Mác thép</t>
   </si>
   <si>
-    <t>Nhóm phân loại</t>
-  </si>
-  <si>
     <t>Thùng số</t>
   </si>
   <si>
     <t>Thời gian</t>
   </si>
   <si>
-    <t>KL thùng LF sau khi ra thép</t>
-  </si>
-  <si>
-    <t>KL thùng &amp; thép lỏng vào bệ xoay (tấn) - lần 1</t>
-  </si>
-  <si>
-    <t>KL thùng (tấn) - lần 2</t>
-  </si>
-  <si>
     <t>KL thùng thép lần 3 (nếu có)</t>
   </si>
   <si>
-    <t>KL thép lỏng (tấn)</t>
-  </si>
-  <si>
     <t>Ghi chú</t>
   </si>
   <si>
     <t>Tinh luyện / Lên thẳng</t>
   </si>
   <si>
-    <t>Phân loại</t>
-  </si>
-  <si>
-    <t>Mác thép BKMIS</t>
-  </si>
-  <si>
-    <t>Thử nghiệm</t>
+    <t>KL thép lỏng (TẤN)</t>
+  </si>
+  <si>
+    <t>KL thùng (TẤN) - lần 2</t>
+  </si>
+  <si>
+    <t>KL thùng &amp; thép lỏng vào Bệ xoay (TẤN) - lần 1</t>
+  </si>
+  <si>
+    <t>Phân loại chất lượng</t>
+  </si>
+  <si>
+    <t>Chúng tôi gồm:
+1. Bên giao: Ông/ Bà:                          Chức vụ:
+2. Bên nhận: Ông/ Bà:                                 Chức vụ:
+Cùng nhau thống nhất lập "Biên Bản giao nhận thép lỏng" chi tiết như sau:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,12 +86,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -108,7 +114,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -131,17 +137,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -172,8 +200,8 @@
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>885826</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>187615</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>568615</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -472,90 +500,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:T4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="16.42578125" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" customWidth="1"/>
-    <col min="15" max="15" width="13.140625" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" customWidth="1"/>
-    <col min="18" max="18" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="19.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="21.85546875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="17.140625" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:20" ht="45.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:20" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="1" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+    </row>
+    <row r="2" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" spans="1:16" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+    </row>
+    <row r="4" spans="1:16" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="L4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="N4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T4" s="1"/>
+      <c r="P4" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>